<commit_message>
test: add basic UI tests for Juice Shop and map them to test cases
</commit_message>
<xml_diff>
--- a/JuiceShop Test-Cases.xlsx
+++ b/JuiceShop Test-Cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KATUDUS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E8AC848-6DCF-47D9-A335-7C8EE262EB1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9711B444-B2A7-4B5A-8AF1-8E64302B4782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="124">
   <si>
     <t>ID</t>
   </si>
@@ -50,16 +50,47 @@
   </si>
   <si>
     <t>Init (Popups)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Popups are shown again until confirmed and are not shown after being dismissed
+Technique: Negative, Positive, State transitions, Use case</t>
+    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
 2 New browser context (no cookies, no local storage)</t>
   </si>
   <si>
+    <t>1 Open http://localhost:3000
+2 Press Escape
+3 Reload the page
+4 Click button "Dismiss"
+5 Reload the page without clicking "Me want it!"
+6 Click button "Me want it!"
+7 Reload the page
+8 Click button "Open Sidenav"</t>
+  </si>
+  <si>
+    <t>Step 1: heading "Welcome to OWASP Juice Shop!" is visible
+Step 2: heading "Welcome to OWASP Juice Shop!" is not visible; cookie "welcomebanner_status" is not set
+Step 3: heading "Welcome to OWASP Juice Shop!" is visible again
+Step 4: heading "Welcome to OWASP Juice Shop!" is not visible; cookie "welcomebanner_status" = "dismiss"; cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is visible
+Step 5: cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is visible; cookie "cookieconsent_status" is not set
+Step 6: cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is not visible; cookie "cookieconsent_status" = "dismiss"
+Step 7: heading "Welcome to OWASP Juice Shop!" and cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." are not visible
+Step 8: side menu is opened; heading "OWASP Juice Shop" is visible</t>
+  </si>
+  <si>
     <t>High</t>
-  </si>
-  <si>
-    <t>+</t>
   </si>
   <si>
     <t>TC-002</t>
@@ -267,53 +298,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">1 Juice Shop is running at http://localhost:3000
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">2 New browser context (no cookies, no local storage)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">3 Welcome Banner and cookie banner are dismissed
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">4 Login page is opened (Account &gt; Login)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>5 User qa.user@juice.test is registered (TC-005)</t>
-    </r>
-  </si>
-  <si>
-    <t>1 Fill "Email" with "qa.user@juice.test", "Password" with "WrongPass123!", click button "Log in"
-2 Fill "Email" with "not.registered@juice.test", "Password" with "Test@12345", click button "Log in"
-3 Fill "Email" with "qa.user", "Password" with "Test@12345", click button "Log in"</t>
-  </si>
-  <si>
     <t>Step 1: Text "Invalid email or password." is visible; URL contains "/#/login"; cookie "token" is not set
 Step 2: Text "Invalid email or password." is visible; URL contains "/#/login"; cookie "token" is not set
 Step 3: Text "Invalid email or password." is visible; URL contains "/#/login"; cookie "token" is not set</t>
@@ -345,12 +329,6 @@
 4 Login page is opened (Account &gt; Login)</t>
   </si>
   <si>
-    <t>1 Email empty, Password empty
-2 Email = "qa.user@juice.test", Password empty
-3 Email empty, Password = "Test@12345"
-4 Email = "qa.user@juice.test", Password = "Test@12345"</t>
-  </si>
-  <si>
     <t>Step 1: button "Log in" is disabled
 Step 2: button "Log in" is disabled
 Step 3: button "Log in" is disabled
@@ -375,22 +353,6 @@
       <t xml:space="preserve">
 Technique: Positive, Use case, State transitions</t>
     </r>
-  </si>
-  <si>
-    <t>1 Fill "Email" with "qa.user@juice.test"
-2 Fill "Password" with "Test@12345"
-3 Click button "Log in"
-4 Click button "Account"
-5 Click menu item "Logout"
-6 Click button "Account"</t>
-  </si>
-  <si>
-    <t>Step 1: field "Email" contains "qa.user@juice.test"
-Step 2: field "Password" is filled, the value is masked
-Step 3: URL contains "/#/search"; cookie "token" is set
-Step 4: menu item "Logout" is visible
-Step 5: cookie "token" is not set; URL does not contain "/#/search"
-Step 6: menu item "Login" is visible; menu item "Logout" is not visible</t>
   </si>
   <si>
     <t>TC-010</t>
@@ -728,7 +690,7 @@
 2 Click button "Your Basket"</t>
   </si>
   <si>
-    <t>Step 1: Snackbar "Added another Apple Juice (1000ml) to basket." is visible; basket counter shows "2"
+    <t>Step 1: Snackbar "Placed Apple Juice (1000ml) into basket." is visible (for a guest the same message is shown again); basket counter shows "2"
 Step 2: Exactly 1 row with "Apple Juice (1000ml)"; quantity "2"; text "Total Price: 3.98¤" is visible</t>
   </si>
   <si>
@@ -854,43 +816,70 @@
 Step 8: Heading contains "Your Basket" and "qa.user@juice.test"; exactly 3 rows: 1st, 2nd and last products of the catalog, each with quantity "1" and the saved price; Total Price = sum of the 3 saved prices with exactly 2 decimal places (e.g. 1.99 + 1.99 + 2.99 -&gt; "Total Price: 6.97¤")</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t>Popups are shown again until confirmed and are not shown after being dismissed
-Technique: Negative, Positive, State transitions, Use case</t>
-    </r>
-  </si>
-  <si>
-    <t>1 Open http://localhost:3000
-2 Press Escape
-3 Reload the page
-4 Click button "Dismiss"
-5 Reload the page without clicking "Me want it!"
-6 Click button "Me want it!"
-7 Reload the page</t>
-  </si>
-  <si>
-    <t>Step 1: heading "Welcome to OWASP Juice Shop!" is visible
-Step 2: heading "Welcome to OWASP Juice Shop!" is not visible; cookie "welcomebanner_status" is not set
-Step 3: heading "Welcome to OWASP Juice Shop!" is visible again
-Step 4: heading "Welcome to OWASP Juice Shop!" is not visible; cookie "welcomebanner_status" = "dismiss"; cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is visible
-Step 5: cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is visible; cookie "cookieconsent_status" is not set
-Step 6: cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is not visible; cookie "cookieconsent_status" = "dismiss"
-Step 7: heading "Welcome to OWASP Juice Shop!" and cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." are not visible; text "OWASP Juice Shop" in the top toolbar is visible</t>
+    <t>tests/juice-shop/init.spec.js › Init (Popups) › Popups are shown again until confirmed and are not shown after being dismissed</t>
+  </si>
+  <si>
+    <t>1 Juice Shop is running at http://localhost:3000
+2 New browser context (no cookies, no local storage)
+3 Welcome Banner and cookie banner are dismissed
+4 Login page is opened (Account &gt; Login)
+5 Built-in user admin@juice-sh.op / admin123 exists</t>
+  </si>
+  <si>
+    <t>1 Fill "Email" with "admin@juice-sh.op", "Password" with "WrongPass123!", click button "Log in"
+2 Fill "Email" with "not.registered@juice.test", "Password" with "Test@12345", click button "Log in"
+3 Fill "Email" with "qa.user", "Password" with "Test@12345", click button "Log in"</t>
+  </si>
+  <si>
+    <t>1 Email empty, Password empty
+2 Email = "admin@juice-sh.op", Password empty
+3 Email empty, Password = "admin123"
+4 Email = "admin@juice-sh.op", Password = "admin123"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Juice Shop is running at http://localhost:3000
+2 New browser context (no cookies, no local storage)
+3 Welcome Banner and cookie banner are dismissed
+4 Login page is opened (Account &gt; Login)
+5 Built-in user admin@juice-sh.op / admin123 exists </t>
+  </si>
+  <si>
+    <t>1 Fill "Email" with "admin@juice-sh.op"
+2 Fill "Password" with "admin123"
+3 Click button "Log in"
+4 Click button "Account"
+5 Click menu item "Logout"
+6 Click button "Account"</t>
+  </si>
+  <si>
+    <t>Step 1: field "Email" contains "admin@juice-sh.op"
+Step 2: field "Password" is filled, the value is masked
+Step 3: URL contains "/#/search"; cookie "token" is set
+Step 4: menu item "Logout" is visible
+Step 5: cookie "token" is not set; URL does not contain "/#/search"
+Step 6: menu item "Login" is visible; menu item "Logout" is not visible</t>
+  </si>
+  <si>
+    <t>tests/juice-shop/login.spec.js › Login › Login with wrong password
+(automated: step 1 - error message and URL; steps 2-3 - manual)</t>
+  </si>
+  <si>
+    <t>tests/juice-shop/login.spec.js › Login › Login with empty email
+(automated: step 3; steps 1, 2, 4 - manual)</t>
+  </si>
+  <si>
+    <t>tests/juice-shop/login.spec.js › Login › Login with valid email
+(automated: steps 1-3 - URL after login; cookie and logout steps 4-6 - manual)</t>
+  </si>
+  <si>
+    <t>tests/juice-shop/products.spec.js › Products › Add a product to the basket and verify it in the basket</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -927,11 +916,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="204"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="13">
@@ -1031,7 +1015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1074,6 +1058,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1390,7 +1377,7 @@
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="52" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="42" customWidth="1"/>
+    <col min="8" max="8" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
@@ -1419,7 +1406,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="208.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" ht="259.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
@@ -1427,176 +1414,176 @@
         <v>9</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>116</v>
+        <v>10</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>117</v>
+        <v>12</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>118</v>
+        <v>13</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H3" s="14"/>
     </row>
     <row r="4" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>21</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>19</v>
       </c>
       <c r="H4" s="14"/>
     </row>
     <row r="5" spans="1:8" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H5" s="14"/>
     </row>
     <row r="6" spans="1:8" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="14"/>
+      <c r="H6" s="15"/>
     </row>
     <row r="7" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H7" s="14"/>
     </row>
     <row r="8" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>41</v>
+        <v>114</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>42</v>
+        <v>115</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>43</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="93.3" customHeight="1" x14ac:dyDescent="0.45">
+        <v>14</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
         <v>44</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>45</v>
@@ -1605,367 +1592,357 @@
         <v>46</v>
       </c>
       <c r="E9" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="F9" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="13" t="s">
-        <v>48</v>
-      </c>
       <c r="G9" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>12</v>
+        <v>21</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>50</v>
-      </c>
       <c r="D10" s="13" t="s">
-        <v>41</v>
+        <v>117</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>51</v>
+        <v>118</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>52</v>
+        <v>119</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="93.3" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>46</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H11" s="14"/>
     </row>
     <row r="12" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="13" t="s">
+      <c r="F12" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>61</v>
-      </c>
       <c r="G12" s="8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H12" s="14"/>
     </row>
     <row r="13" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="B13" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>65</v>
-      </c>
       <c r="G13" s="10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H13" s="14"/>
     </row>
     <row r="14" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="E14" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="F14" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>71</v>
-      </c>
       <c r="G14" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>12</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H14" s="15"/>
     </row>
     <row r="15" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>75</v>
-      </c>
       <c r="G15" s="8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H15" s="14"/>
     </row>
     <row r="16" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C16" s="13" t="s">
+      <c r="G16" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>80</v>
       </c>
       <c r="H16" s="14"/>
     </row>
     <row r="17" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="F17" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>84</v>
-      </c>
       <c r="G17" s="8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H17" s="14"/>
     </row>
     <row r="18" spans="1:8" ht="157.05000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="E18" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="F18" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="D18" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>90</v>
-      </c>
       <c r="G18" s="8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H18" s="14"/>
     </row>
     <row r="19" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" s="13" t="s">
+      <c r="F19" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="D19" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>95</v>
-      </c>
       <c r="G19" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H19" s="14" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E20" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="B20" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" s="13" t="s">
+      <c r="F20" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="F20" s="13" t="s">
-        <v>100</v>
-      </c>
       <c r="G20" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>12</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="H20" s="15"/>
     </row>
     <row r="21" spans="1:8" ht="144.30000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="B21" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="13" t="s">
+      <c r="F21" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="D21" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>105</v>
-      </c>
       <c r="G21" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>12</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="H21" s="15"/>
     </row>
     <row r="22" spans="1:8" ht="144.30000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C22" s="13" t="s">
+      <c r="F22" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="D22" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>110</v>
-      </c>
       <c r="G22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>12</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H22" s="15"/>
     </row>
     <row r="23" spans="1:8" ht="208.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="E23" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="13" t="s">
+      <c r="F23" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="D23" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>115</v>
-      </c>
       <c r="G23" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>12</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H23" s="15"/>
     </row>
     <row r="24" spans="1:8" ht="208.05" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>

</xml_diff>

<commit_message>
test: add more UI tests based on the test cases
</commit_message>
<xml_diff>
--- a/JuiceShop Test-Cases.xlsx
+++ b/JuiceShop Test-Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KATUDUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\INNOWISE\AQA intern\AQA\ДЗ №3-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9711B444-B2A7-4B5A-8AF1-8E64302B4782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E5D617-CFDF-4AFF-8A43-513FCAC8860F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="21795" windowHeight="11625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="125">
   <si>
     <t>ID</t>
   </si>
@@ -52,18 +52,8 @@
     <t>Init (Popups)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t>Popups are shown again until confirmed and are not shown after being dismissed
+    <t>Popups are shown again until confirmed and are not shown after being dismissed
 Technique: Negative, Positive, State transitions, Use case</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
@@ -86,34 +76,24 @@
 Step 4: heading "Welcome to OWASP Juice Shop!" is not visible; cookie "welcomebanner_status" = "dismiss"; cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is visible
 Step 5: cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is visible; cookie "cookieconsent_status" is not set
 Step 6: cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." is not visible; cookie "cookieconsent_status" = "dismiss"
-Step 7: heading "Welcome to OWASP Juice Shop!" and cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." are not visible
+Step 7: heading "Welcome to OWASP Juice Shop!" and cookie banner text "This website uses fruit cookies to ensure you get the juiciest tracking experience." are not visible; basket counter shows "0"
 Step 8: side menu is opened; heading "OWASP Juice Shop" is visible</t>
   </si>
   <si>
     <t>High</t>
   </si>
   <si>
+    <t>init.spec.js</t>
+  </si>
+  <si>
     <t>TC-002</t>
   </si>
   <si>
     <t>Registration</t>
   </si>
   <si>
-    <r>
-      <t>Navigation Login &lt;-&gt; Registration</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Navigation Login &lt;-&gt; Registration
 Technique: Positive, State transitions</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
@@ -136,24 +116,14 @@
     <t>Medium</t>
   </si>
   <si>
+    <t>registration.spec.js</t>
+  </si>
+  <si>
     <t>TC-003</t>
   </si>
   <si>
-    <r>
-      <t>Registration form shows validation errors for invalid data</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Registration form shows validation errors for invalid data
 Technique: Negative, Equivalence classes (invalid email), Boundary values (password length)</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
@@ -179,21 +149,8 @@
     <t>TC-004</t>
   </si>
   <si>
-    <r>
-      <t>"Register" button state when a required field is empty</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>"Register" button state when a required field is empty
 Technique: Negative, Condition overlay (decision table)</t>
-    </r>
   </si>
   <si>
     <t>1 All fields empty
@@ -211,30 +168,17 @@
     <t>TC-005</t>
   </si>
   <si>
-    <r>
-      <t>Register with valid data</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Register with valid data
 Technique: Positive, Use case</t>
-    </r>
-  </si>
-  <si>
-    <t>1 Fill "Email" with "qa.user@juice.test"
+  </si>
+  <si>
+    <t>1 Fill "Email" with a valid email that is not registered yet
 2 Fill "Password" and "Repeat Password" with "Test@12345"
 3 Select the 1st option in "Security Question", fill "Answer" with "Test"
 4 Click button "Register"</t>
   </si>
   <si>
-    <t>Step 1: field "Email" contains "qa.user@juice.test"
+    <t>Step 1: field "Email" contains the entered email
 Step 2: fields "Password" and "Repeat Password" are filled, the values are masked; no error message is shown
 Step 3: the selected question is shown in "Security Question"; field "Answer" contains "Test"
 Step 4: Snackbar "Registration completed successfully. You can now log in." is visible; URL contains "/#/login"</t>
@@ -243,31 +187,18 @@
     <t>TC-006</t>
   </si>
   <si>
-    <r>
-      <t>Register with an already registered email</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Register with an already registered email
 Technique: Negative</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
 2 New browser context (no cookies, no local storage)
 3 Welcome Banner and cookie banner are dismissed
 4 Registration page is opened (Account &gt; Login &gt; "Not yet a customer?")
-5 User qa.user@juice.test is already registered</t>
-  </si>
-  <si>
-    <t>1 Fill all fields with valid data, "Email" = "qa.user@juice.test"
+5 User is already registered</t>
+  </si>
+  <si>
+    <t>1 Fill all fields with valid data, "Email" = the email of the registered user
 2 Click button "Register"</t>
   </si>
   <si>
@@ -281,21 +212,20 @@
     <t>Login</t>
   </si>
   <si>
-    <r>
-      <t>Login with invalid credentials</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Login with invalid credentials
 Technique: Negative, Equivalence classes (wrong password, non-existing user, invalid email format)</t>
-    </r>
+  </si>
+  <si>
+    <t>1 Juice Shop is running at http://localhost:3000
+2 New browser context (no cookies, no local storage)
+3 Welcome Banner and cookie banner are dismissed
+4 Login page is opened (Account &gt; Login)
+5 Built-in user admin@juice-sh.op / admin123 exists</t>
+  </si>
+  <si>
+    <t>1 Fill "Email" with "admin@juice-sh.op", "Password" with "WrongPass123!", click button "Log in"
+2 Fill "Email" with "not.registered@juice.test", "Password" with "Test@12345", click button "Log in"
+3 Fill "Email" with "qa.user", "Password" with "Test@12345", click button "Log in"</t>
   </si>
   <si>
     <t>Step 1: Text "Invalid email or password." is visible; URL contains "/#/login"; cookie "token" is not set
@@ -303,24 +233,14 @@
 Step 3: Text "Invalid email or password." is visible; URL contains "/#/login"; cookie "token" is not set</t>
   </si>
   <si>
+    <t>login.spec.js</t>
+  </si>
+  <si>
     <t>TC-008</t>
   </si>
   <si>
-    <r>
-      <t>"Log in" button state for empty / filled fields</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>"Log in" button state for empty / filled fields
 Technique: Negative, Condition overlay (decision table)</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
@@ -329,6 +249,12 @@
 4 Login page is opened (Account &gt; Login)</t>
   </si>
   <si>
+    <t>1 Email empty, Password empty
+2 Email = "admin@juice-sh.op", Password empty
+3 Email empty, Password = "admin123"
+4 Email = "admin@juice-sh.op", Password = "admin123"</t>
+  </si>
+  <si>
     <t>Step 1: button "Log in" is disabled
 Step 2: button "Log in" is disabled
 Step 3: button "Log in" is disabled
@@ -338,41 +264,38 @@
     <t>TC-009</t>
   </si>
   <si>
-    <r>
-      <t>Login with valid email and password, then logout</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Login with valid email and password, then logout
 Technique: Positive, Use case, State transitions</t>
-    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Juice Shop is running at http://localhost:3000
+2 New browser context (no cookies, no local storage)
+3 Welcome Banner and cookie banner are dismissed
+4 Login page is opened (Account &gt; Login)
+5 Built-in user admin@juice-sh.op / admin123 exists </t>
+  </si>
+  <si>
+    <t>1 Fill "Email" with "admin@juice-sh.op"
+2 Fill "Password" with "admin123"
+3 Click button "Log in"
+4 Click button "Account"
+5 Click menu item "Logout"
+6 Click button "Account"</t>
+  </si>
+  <si>
+    <t>Step 1: field "Email" contains "admin@juice-sh.op"
+Step 2: field "Password" is filled, the value is masked
+Step 3: URL contains "/#/search"; cookie "token" is set
+Step 4: menu item "Logout" is visible
+Step 5: cookie "token" is not set; URL does not contain "/#/search"
+Step 6: menu item "Login" is visible; menu item "Logout" is not visible</t>
   </si>
   <si>
     <t>TC-010</t>
   </si>
   <si>
-    <r>
-      <t>Forgot password: page opens, fields stay disabled for an unregistered email</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Forgot password: page opens, fields stay disabled for an unregistered email
 Technique: Negative, State transitions</t>
-    </r>
   </si>
   <si>
     <t>1 Click link "Forgot your password?"
@@ -383,38 +306,28 @@
 Step 2: Fields "Security Question", "New Password", "Repeat New Password" stay disabled; button "Change" is disabled</t>
   </si>
   <si>
+    <t>manually</t>
+  </si>
+  <si>
     <t>TC-011</t>
   </si>
   <si>
-    <r>
-      <t>Forgot password: new passwords do not match, wrong answer to the security question</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Forgot password: new passwords do not match, wrong answer to the security question
 Technique: Negative</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
 2 New browser context (no cookies, no local storage)
 3 Welcome Banner and cookie banner are dismissed
-4 User reset.user@juice.test / Test@12345 is registered, security answer "Test"
+4 User is registered with password "Test@12345" and security answer "Test"
 5 Forgot Password page is opened (Account &gt; Login &gt; "Forgot your password?")</t>
   </si>
   <si>
-    <t>1 Fill "Email" with "reset.user@juice.test"
+    <t>1 Fill "Email" with the email of the registered user
 2 Fill "Security Question" with "Test", "New Password" with "NewPass@123", "Repeat New Password" with "NewPass@321"
 3 Change "Security Question" to "WrongAnswer" and "Repeat New Password" to "NewPass@123"
 4 Click button "Change"
-5 Open Login page, log in with reset.user@juice.test / Test@12345 (old password)</t>
+5 Open Login page, log in with the email of the registered user and "Test@12345" (old password)</t>
   </si>
   <si>
     <t>Step 1: fields "Security Question", "New Password", "Repeat New Password" become enabled
@@ -427,27 +340,14 @@
     <t>TC-012</t>
   </si>
   <si>
-    <r>
-      <t>Forgot password: change password and log in with the new one</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Forgot password: change password and log in with the new one
 Technique: Positive, State transitions</t>
-    </r>
-  </si>
-  <si>
-    <t>1 Fill "Email" with "reset.user@juice.test", "Security Question" with "Test", "New Password" and "Repeat New Password" with "NewPass@123"
+  </si>
+  <si>
+    <t>1 Fill "Email" with the email of the registered user, "Security Question" with "Test", "New Password" and "Repeat New Password" with "NewPass@123"
 2 Click button "Change"
-3 Open Login page, log in with reset.user@juice.test / Test@12345 (old password)
-4 Log in with reset.user@juice.test / NewPass@123 (new password)</t>
+3 Open Login page, log in with the email of the registered user and "Test@12345" (old password)
+4 Log in with the email of the registered user and "NewPass@123" (new password)</t>
   </si>
   <si>
     <t>Step 1: button "Change" is enabled
@@ -462,27 +362,14 @@
     <t>Products</t>
   </si>
   <si>
-    <r>
-      <t>Product list is displayed</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Product list is displayed
 Technique: Positive</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
 2 New browser context (no cookies, no local storage)
 3 Welcome Banner and cookie banner are dismissed
-4 User qa.user@juice.test / Test@12345 is registered and logged in
+4 User is registered and logged in
 5 All Products page (/#/search) is opened</t>
   </si>
   <si>
@@ -492,21 +379,14 @@
     <t>Step 1: Title "All Products" is visible; number of product cards &gt; 0; every card contains a price with "¤" and button "Add to Basket"</t>
   </si>
   <si>
+    <t>products.spec.js</t>
+  </si>
+  <si>
     <t>TC-014</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t>Pagination: first and last page, "Items per page" options
+    <t>Pagination: first and last page, "Items per page" options
 Technique: Boundary values, Equivalence classes</t>
-    </r>
   </si>
   <si>
     <t>1 Read the selected value N in "Items per page" and the total T from the counter "1 – N of T"
@@ -524,21 +404,8 @@
     <t>TC-015</t>
   </si>
   <si>
-    <r>
-      <t>Search for a non-existing product</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Search for a non-existing product
 Technique: Negative</t>
-    </r>
   </si>
   <si>
     <t>1 Click the search icon
@@ -555,21 +422,8 @@
     <t>TC-016</t>
   </si>
   <si>
-    <r>
-      <t>Search by full product name and by part of the name in lower case</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Search by full product name and by part of the name in lower case
 Technique: Positive, Equivalence classes (exact name; partial, case-insensitive)</t>
-    </r>
   </si>
   <si>
     <t>1 Click the search icon
@@ -588,27 +442,14 @@
     <t>Basket</t>
   </si>
   <si>
-    <r>
-      <t>Sold-out product cannot be added</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Sold-out product cannot be added
 Technique: Negative</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
 2 New browser context (no cookies, no local storage)
 3 Welcome Banner and cookie banner are dismissed
-4 User is NOT logged in
+4 User is registered and logged in
 5 All Products page (/#/search) is opened
 6 Basket is empty
 7 A product card with the "Sold Out" label exists</t>
@@ -618,28 +459,15 @@
 2 Click button "Your Basket"</t>
   </si>
   <si>
-    <t>Step 1: snackbar "We are out of stock! Sorry for the inconvenience." is visible
+    <t>Step 1: snackbar "We are out of stock! Sorry for the inconvenience." is visible; basket counter shows "0"
 Step 2: 0 rows; text "Total Price: 0¤" is visible</t>
   </si>
   <si>
     <t>TC-018</t>
   </si>
   <si>
-    <r>
-      <t>Add a product to the basket and verify it in the basket</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Add a product to the basket and verify it in the basket
 Technique: Positive, Use case</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
@@ -658,24 +486,14 @@
 Step 2: heading contains "Your Basket" and "(anonymous)"; URL contains "/#/basket"; exactly 1 row; row contains "Apple Juice (1000ml)", quantity "1", price "1.99¤"; text "Total Price: 1.99¤" is visible</t>
   </si>
   <si>
+    <t>basket.spec.js</t>
+  </si>
+  <si>
     <t>TC-019</t>
   </si>
   <si>
-    <r>
-      <t>Add the same product again: the quantity is summed</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Add the same product again: the quantity is summed
 Technique: State transitions</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
@@ -697,21 +515,8 @@
     <t>TC-020</t>
   </si>
   <si>
-    <r>
-      <t>Change the quantity with "-" and "+": not below 1</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Change the quantity with "-" and "+": not below 1
 Technique: Negative, Boundary values, State transitions</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
@@ -736,21 +541,8 @@
     <t>TC-021</t>
   </si>
   <si>
-    <r>
-      <t>Delete the product: the basket becomes empty</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
+    <t>Delete the product: the basket becomes empty
 Technique: State transitions</t>
-    </r>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
@@ -771,115 +563,39 @@
     <t>TC-022</t>
   </si>
   <si>
-    <r>
-      <t>Guest basket is kept after reload and merged into the user basket after login; total price</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
-Technique: State transitions, Boundary values (1st and last product), Use case</t>
-    </r>
+    <t>Guest basket is merged into the user basket after login
+Technique: State transitions, Use case</t>
   </si>
   <si>
     <t>1 Juice Shop is running at http://localhost:3000
 2 New browser context (no cookies, no local storage)
 3 Welcome Banner and cookie banner are dismissed
-4 User qa.user@juice.test / Test@12345 is registered
+4 User is registered
 5 User is NOT logged in; the user basket is empty
 6 All Products page (/#/search) is opened</t>
   </si>
   <si>
-    <t>1 Click button "Account", click menu item "Login", log in with qa.user@juice.test / Test@12345
-2 Click "Add to Basket" on the 2nd card of page 1; save its name and price
+    <t>1 Click button "Account", click menu item "Login", log in with the email and password of the registered user
+2 Click "Add to Basket" on the "Apple Juice (1000ml)" card
 3 Click button "Account", click menu item "Logout"
-4 Click "Add to Basket" on the 1st card of page 1; save its name and price
-5 Click "Add to Basket" on the LAST card of the catalog; save its name and price
-6 Reload the page, click button "Your Basket"
-7 Click button "Account", click menu item "Login", log in with qa.user@juice.test / Test@12345
-8 Click button "Your Basket"</t>
+4 Click "Add to Basket" on the "Banana Juice (1000ml)" card
+5 Click button "Account", click menu item "Login", log in with the same user
+6 Click button "Your Basket"</t>
   </si>
   <si>
     <t>Step 1: URL contains "/#/search"; cookie "token" is set
-Step 2: snackbar "Placed &lt;name&gt; into basket." is visible; basket counter shows "1"
-Step 3: cookie "token" is not set
-Step 4: snackbar "Placed &lt;name&gt; into basket." is visible
-Step 5: snackbar "Placed &lt;name&gt; into basket." is visible
-Step 6: exactly 2 rows: 1st and last products with quantity "1" and the saved prices; Total Price = sum of the 2 saved prices with exactly 2 decimal places
-Step 7: URL contains "/#/search"; cookie "token" is set
-Step 8: Heading contains "Your Basket" and "qa.user@juice.test"; exactly 3 rows: 1st, 2nd and last products of the catalog, each with quantity "1" and the saved price; Total Price = sum of the 3 saved prices with exactly 2 decimal places (e.g. 1.99 + 1.99 + 2.99 -&gt; "Total Price: 6.97¤")</t>
-  </si>
-  <si>
-    <t>tests/juice-shop/init.spec.js › Init (Popups) › Popups are shown again until confirmed and are not shown after being dismissed</t>
-  </si>
-  <si>
-    <t>1 Juice Shop is running at http://localhost:3000
-2 New browser context (no cookies, no local storage)
-3 Welcome Banner and cookie banner are dismissed
-4 Login page is opened (Account &gt; Login)
-5 Built-in user admin@juice-sh.op / admin123 exists</t>
-  </si>
-  <si>
-    <t>1 Fill "Email" with "admin@juice-sh.op", "Password" with "WrongPass123!", click button "Log in"
-2 Fill "Email" with "not.registered@juice.test", "Password" with "Test@12345", click button "Log in"
-3 Fill "Email" with "qa.user", "Password" with "Test@12345", click button "Log in"</t>
-  </si>
-  <si>
-    <t>1 Email empty, Password empty
-2 Email = "admin@juice-sh.op", Password empty
-3 Email empty, Password = "admin123"
-4 Email = "admin@juice-sh.op", Password = "admin123"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Juice Shop is running at http://localhost:3000
-2 New browser context (no cookies, no local storage)
-3 Welcome Banner and cookie banner are dismissed
-4 Login page is opened (Account &gt; Login)
-5 Built-in user admin@juice-sh.op / admin123 exists </t>
-  </si>
-  <si>
-    <t>1 Fill "Email" with "admin@juice-sh.op"
-2 Fill "Password" with "admin123"
-3 Click button "Log in"
-4 Click button "Account"
-5 Click menu item "Logout"
-6 Click button "Account"</t>
-  </si>
-  <si>
-    <t>Step 1: field "Email" contains "admin@juice-sh.op"
-Step 2: field "Password" is filled, the value is masked
-Step 3: URL contains "/#/search"; cookie "token" is set
-Step 4: menu item "Logout" is visible
-Step 5: cookie "token" is not set; URL does not contain "/#/search"
-Step 6: menu item "Login" is visible; menu item "Logout" is not visible</t>
-  </si>
-  <si>
-    <t>tests/juice-shop/login.spec.js › Login › Login with wrong password
-(automated: step 1 - error message and URL; steps 2-3 - manual)</t>
-  </si>
-  <si>
-    <t>tests/juice-shop/login.spec.js › Login › Login with empty email
-(automated: step 3; steps 1, 2, 4 - manual)</t>
-  </si>
-  <si>
-    <t>tests/juice-shop/login.spec.js › Login › Login with valid email
-(automated: steps 1-3 - URL after login; cookie and logout steps 4-6 - manual)</t>
-  </si>
-  <si>
-    <t>tests/juice-shop/products.spec.js › Products › Add a product to the basket and verify it in the basket</t>
+Step 2: snackbar "Placed Apple Juice (1000ml) into basket." is visible; basket counter shows "1"
+Step 3: cookie "token" is not set; basket counter shows "0"
+Step 4: snackbar "Placed Banana Juice (1000ml) into basket." is visible; basket counter shows "1"
+Step 5: URL contains "/#/search"; cookie "token" is set; basket counter shows "2"
+Step 6: heading contains "Your Basket" and the email of the user; exactly 2 rows: "Apple Juice (1000ml)" and "Banana Juice (1000ml)", each with quantity "1"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -904,14 +620,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -1015,7 +723,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1058,9 +766,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1406,7 +1111,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="259.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" ht="270.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
@@ -1428,521 +1133,555 @@
       <c r="G2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="15" t="s">
-        <v>113</v>
+      <c r="H2" s="14" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="14"/>
+        <v>22</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="13" t="s">
+      <c r="H4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" s="14"/>
     </row>
     <row r="5" spans="1:8" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" s="14"/>
+        <v>22</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="15"/>
+      <c r="H6" s="14" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="14"/>
+        <v>22</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>114</v>
+        <v>45</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>115</v>
+        <v>46</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="15" t="s">
-        <v>120</v>
+      <c r="H8" s="14" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="106.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>116</v>
+        <v>52</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" s="15" t="s">
-        <v>121</v>
+        <v>22</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>117</v>
+        <v>56</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>118</v>
+        <v>57</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>119</v>
+        <v>58</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="15" t="s">
-        <v>122</v>
+      <c r="H10" s="14" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="93.3" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="13" t="s">
-        <v>46</v>
-      </c>
       <c r="E11" s="13" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H11" s="14"/>
+        <v>22</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" s="14"/>
+        <v>22</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="14"/>
+      <c r="H13" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="15"/>
+      <c r="H14" s="14" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="4" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H15" s="14"/>
+        <v>22</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="H16" s="14"/>
+        <v>88</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="118.8" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H17" s="14"/>
+        <v>22</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="157.05000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="4" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H18" s="14"/>
+        <v>22</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="4" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="G19" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="15" t="s">
-        <v>123</v>
+      <c r="H19" s="14" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="131.55000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" s="15"/>
+        <v>22</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="144.30000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H21" s="15"/>
+        <v>22</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="144.30000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="4" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H22" s="15"/>
+      <c r="H22" s="14" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="208.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="G23" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H23" s="15"/>
+      <c r="H23" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="24" spans="1:8" ht="208.05" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>

</xml_diff>